<commit_message>
fix: fixed bugs and edited test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-48_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-48_Test_Cases.xlsx
@@ -28,15 +28,6 @@
     <sheet name="TC19" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="TC20" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="TC21" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="TC22" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="TC23" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="TC24" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="TC25" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="TC26" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="TC27" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="TC28" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="TC29" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="TC30" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -45,8 +36,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -479,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -506,7 +498,6 @@
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="9" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -552,17 +543,17 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Availability check matches on the requested equipment type</t>
+          <t>Equipment type with no stock at all is reported as unavailable</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>AC1</t>
+          <t>AC1, AC2</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F4" s="11" t="inlineStr">
@@ -584,17 +575,17 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Equipment type with no stock at all is reported as unavailable</t>
+          <t>Requested quantity exactly equal to available stock is sufficient</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC2</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
@@ -616,7 +607,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Sufficient quantity is reported when stock exceeds the request</t>
+          <t>Requested quantity one more than available stock is insufficient</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -626,7 +617,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
@@ -648,7 +639,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Insufficient quantity is reported when the request exceeds stock</t>
+          <t>Requesting zero units is rejected with a validation message</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -663,7 +654,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -680,17 +671,17 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Requested quantity exactly equal to available stock is sufficient</t>
+          <t>Overlapping events competing for the same equipment reduce the available quantity</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC3, AC4</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
@@ -712,22 +703,22 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Requested quantity one more than available stock is insufficient</t>
+          <t>A request that is only requested or under review does not reduce availability</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -744,17 +735,17 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Requesting zero units is rejected with a validation message</t>
+          <t>A partially fulfilled reservation reduces availability by the quantity reserved</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -776,12 +767,12 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Same equipment gives a different result for a different event date</t>
+          <t>Equipment held by a cancelled event is released</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -791,7 +782,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -808,17 +799,17 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Availability is recalculated when the event is rescheduled</t>
+          <t>Equipment is unavailable the day after another event's Return Day</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -840,17 +831,17 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Overlapping events competing for the same equipment reduce the available quantity</t>
+          <t>Equipment is available for an event two days after another event's Return Day</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>AC3, AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F13" s="11" t="inlineStr">
@@ -872,17 +863,17 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Events on unrelated dates do not affect each other's availability</t>
+          <t>A multi-day reservation blocks the equipment until the day after its last day</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -904,22 +895,22 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>A request that is only requested or under review does not reduce availability</t>
+          <t>A late-night finish does not extend the blocked period</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC5, AC6</t>
         </is>
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -936,22 +927,22 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>A partially fulfilled reservation reduces availability by the quantity reserved</t>
+          <t>Two events on the same day cannot share the same single unit, even at different times</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC4, AC5</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -968,12 +959,12 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Equipment held by a cancelled event is released</t>
+          <t>Two events on the same day can both be supported when stock covers both</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC4, AC5</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -983,7 +974,7 @@
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -1000,17 +991,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Equipment is unavailable the day after another event's Return Day</t>
+          <t>Each session of a multi-session event is checked against its own dates</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC3, AC5</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1032,17 +1023,17 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Equipment is available for an event two days after another event's Return Day</t>
+          <t>Equipment in ConnectSphere storage leaves the fixed transfer/prep time before the event</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F19" s="11" t="inlineStr">
@@ -1064,17 +1055,17 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Equipment is unavailable for an event the day before another reservation's collection day</t>
+          <t>No transfer time is added when the equipment is already at the event venue</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
@@ -1096,12 +1087,12 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>A multi-day reservation blocks the equipment until the day after its last day</t>
+          <t>Availability is still shown when the event has no venue yet</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -1128,17 +1119,17 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>A late-night finish does not extend the blocked period</t>
+          <t>Units under maintenance are excluded from the available count</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>AC5, AC6</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -1160,12 +1151,12 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Two events on the same day cannot share the same single unit, even at different times</t>
+          <t>Retired equipment is unavailable on an existing request and hidden from the Add list</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>AC4, AC5</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -1175,7 +1166,7 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1183,12 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Two events on the same day can both be supported when stock covers both</t>
+          <t>A request with several lines shows a result per line and one overall banner</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>AC4, AC5</t>
+          <t>AC2, AC8</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
@@ -1211,513 +1202,213 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>TC22</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC22</t>
-        </is>
-      </c>
-      <c r="C25" s="11" t="inlineStr">
-        <is>
-          <t>Each session of a multi-session event is checked against its own dates</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>AC3, AC5</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>TC23</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC23</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>Equipment in ConnectSphere storage leaves the fixed transfer/prep time before the event</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>TC24</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC24</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>No transfer time is added when the equipment is already at the event venue</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>TC25</t>
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Acceptance Criterion</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="17.5" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>SPM-48-TC25</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>Availability is still shown when the event has no venue yet</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
+          <t>The system considers the required equipment type.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="9" t="n"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>TC26</t>
+          <t>SPM-48-TC01</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="71.5" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>AC2</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>SPM-48-TC26</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="inlineStr">
-        <is>
-          <t>Units under maintenance are excluded from the available count</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
+          <t>The system considers the required quantity.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>TC27</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC27</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Retired equipment is unavailable on an existing request and hidden from the Add list</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>TC28</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC28</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>Sufficient availability is indicated on the line and no shortfall banner is shown</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>AC8</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>TC29</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC29</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>Insufficient availability is indicated with the shortfall and the banner</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>AC8</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>TC30</t>
-        </is>
-      </c>
-      <c r="B33" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC30</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>A request with several lines shows a result per line and one overall banner</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr">
-        <is>
-          <t>AC2, AC8</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="inlineStr">
-        <is>
-          <t>Acceptance Criteria</t>
-        </is>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="7" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="n"/>
-    </row>
-    <row r="37" ht="31" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>The system considers the required equipment type.</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
           <t>SPM-48-TC01
-SPM-48-TC02</t>
-        </is>
-      </c>
-      <c r="F37" s="9" t="n"/>
-    </row>
-    <row r="38" ht="98.5" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>The system considers the required quantity.</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="n"/>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC02
+SPM-48-TC02
 SPM-48-TC03
 SPM-48-TC04
-SPM-48-TC05
+SPM-48-TC21</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="31" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>AC3</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>The system considers the event date and time.</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>SPM-48-TC05
+SPM-48-TC15</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="85" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Equipment already reserved for overlapping events is excluded from available quantities.</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>SPM-48-TC05
 SPM-48-TC06
 SPM-48-TC07
-SPM-48-TC30</t>
-        </is>
-      </c>
-      <c r="F38" s="9" t="n"/>
-    </row>
-    <row r="39" ht="58" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
-        <is>
-          <t>AC3</t>
-        </is>
-      </c>
-      <c r="B39" s="11" t="inlineStr">
-        <is>
-          <t>The system considers the event date and time.</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="n"/>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC08
-SPM-48-TC09
+SPM-48-TC08
+SPM-48-TC13
+SPM-48-TC14</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="98.5" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>AC5</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Equipment is treated as unavailable from its collection day (D-1) through the day after its return (Return Day+1), not only during the event's own date and time.</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>SPM-48-TC09
 SPM-48-TC10
-SPM-48-TC22</t>
-        </is>
-      </c>
-      <c r="F39" s="9" t="n"/>
-    </row>
-    <row r="40" ht="98.5" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B40" s="11" t="inlineStr">
-        <is>
-          <t>Equipment already reserved for overlapping events is excluded from available quantities.</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="n"/>
-      <c r="D40" s="9" t="n"/>
-      <c r="E40" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC10
 SPM-48-TC11
 SPM-48-TC12
 SPM-48-TC13
 SPM-48-TC14
-SPM-48-TC20
-SPM-48-TC21</t>
-        </is>
-      </c>
-      <c r="F40" s="9" t="n"/>
-    </row>
-    <row r="41" ht="112" customHeight="1">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>AC5</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="inlineStr">
-        <is>
-          <t>Equipment is treated as unavailable from its collection day (D-1) through the day after its return (Return Day+1), not only during the event's own date and time.</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="n"/>
-      <c r="D41" s="9" t="n"/>
-      <c r="E41" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC15
+SPM-48-TC15</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="58" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>AC6</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Required transfer and preparation time between the equipment's current location and the event venue is factored into availability.</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>SPM-48-TC12
 SPM-48-TC16
 SPM-48-TC17
-SPM-48-TC18
-SPM-48-TC19
-SPM-48-TC20
-SPM-48-TC21
-SPM-48-TC22</t>
-        </is>
-      </c>
-      <c r="F41" s="9" t="n"/>
-    </row>
-    <row r="42" ht="58" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="inlineStr">
-        <is>
-          <t>Required transfer and preparation time between the equipment's current location and the event venue is factored into availability.</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="11" t="inlineStr">
+SPM-48-TC18</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="31" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Equipment recorded as unavailable is excluded.</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>SPM-48-TC19
-SPM-48-TC23
-SPM-48-TC24
-SPM-48-TC25</t>
-        </is>
-      </c>
-      <c r="F42" s="9" t="n"/>
-    </row>
-    <row r="43" ht="31" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B43" s="11" t="inlineStr">
-        <is>
-          <t>Equipment recorded as unavailable is excluded.</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC26
-SPM-48-TC27</t>
-        </is>
-      </c>
-      <c r="F43" s="9" t="n"/>
-    </row>
-    <row r="44" ht="44.5" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+SPM-48-TC20</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="17.5" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>AC8</t>
         </is>
       </c>
-      <c r="B44" s="11" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>The system indicates whether sufficient equipment is available.</t>
         </is>
       </c>
-      <c r="C44" s="8" t="n"/>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="11" t="inlineStr">
-        <is>
-          <t>SPM-48-TC28
-SPM-48-TC29
-SPM-48-TC30</t>
-        </is>
-      </c>
-      <c r="F44" s="9" t="n"/>
-    </row>
-    <row r="45"/>
-    <row r="46" ht="152.5" customHeight="1">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>SPM-48-TC21</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
+    </row>
+    <row r="37" ht="152.5" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>src/lib/equipment.ts
 prisma/schema.prisma
@@ -1732,33 +1423,33 @@
 src/lib/equipment.ts</t>
         </is>
       </c>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="9" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="B46:F46"/>
-    <mergeCell ref="B44:D44"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="B38:D38"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="B30:D30"/>
     <mergeCell ref="B1:F1"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="B27:D27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1782,15 +1473,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1829,7 +1511,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="206.5" customHeight="1">
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1837,17 +1519,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #16 and #114 (a reschedule or change means availability is re-checked). The change flow (SPM-32 / SPM-35) is not built, so 'Homecoming Weekend' is seeded as if already moved onto 2026-11-10.
-'Follow Spot': 1 total, 0 in maintenance.
-Event 'Faculty Day' (2026-11-10) holds 1x Follow Spot (reserved).
-Event 'Homecoming Weekend' (2026-11-10, 'rescheduled' here) requests 1x Follow Spot.
+          <t>Rule source: customer Q&amp;A #5 (collected one day before the event, available again from Return Day+1). Return Day is the day the event ends.
+'Lighting Rig': 1 total, 0 in maintenance.
+Event 'Gala Dinner' (Monday 2026-11-02, 10:00-16:00) holds 1x Lighting Rig: blocked from its D-1 (2026-11-01) through its Return Day (2026-11-02).
+Event 'Charity Concert' (Tuesday 2026-11-03) requests 1x Lighting Rig. It would need collecting on 2026-11-02 (its own D-1), while the rig is still being returned and checked.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1856,8 +1538,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Homecoming Weekend event
-3. Read the Follow Spot line under Requested items</t>
+2. Open the equipment request for the Charity Concert event
+3. Read the Lighting Rig line under Requested items</t>
         </is>
       </c>
     </row>
@@ -1869,11 +1551,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Follow Spot, Requested: 1, New event date: 2026-11-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>Equipment: Lighting Rig, Requested: 1, Checked date: 2026-11-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1881,8 +1563,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Follow Spot line reflects the new date: chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
-The line notes 'Held by Faculty Day (1 unit) until 11 Nov.'
+          <t>The Lighting Rig line shows the chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
+The line notes 'Held by Gala Dinner (1 unit) until 3 Nov.' (the day it is available again, Return Day+1).
 The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
@@ -1909,7 +1591,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -1927,7 +1608,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Follow Spot line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Faculty Day (1 unit) until 11 Nov. Venue not yet chosen — transfer time not included.
+          <t>Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Gala Dinner (1 unit) until 3 Nov. Venue not yet chosen — transfer time not included.
 Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
@@ -1952,7 +1633,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. The event is seeded as already rescheduled: the change flow (SPM-32 / SPM-35) is not built.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
         </is>
       </c>
     </row>
@@ -2024,16 +1705,16 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'HD Projector': 3 total, 0 in maintenance.
-Event 'Board Meeting' (2026-10-26, 10:00-12:00) holds 2x HD Projector (reserved).
-Event 'Investor Briefing' (2026-10-26, 11:00-13:00, overlapping Board Meeting) requests 2x HD Projector.
+          <t>'Lighting Rig': 1 total, 0 in maintenance.
+Event 'Gala Dinner' (Monday 2026-11-02) holds 1x Lighting Rig; it is available again from Return Day+1 (2026-11-03).
+Event 'School Concert' (Wednesday 2026-11-04) requests 1x Lighting Rig; its own D-1 is 2026-11-03.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2042,8 +1723,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Investor Briefing event
-3. Read the HD Projector line under Requested items</t>
+2. Open the equipment request for the School Concert event
+3. Read the Lighting Rig line under Requested items</t>
         </is>
       </c>
     </row>
@@ -2055,11 +1736,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: HD Projector, Requested: 2, Total: 3, Reserved by overlapping event: 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Equipment: Lighting Rig, Requested: 1, Checked date: 2026-11-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2067,9 +1748,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The HD Projector line shows the chip 'Partial', '3 total − 0 in maintenance − 2 reserved elsewhere = 1 available for these dates' and '2 requested, 1 available.'
-The 2 units held by Board Meeting are excluded from the available count.
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -2095,7 +1775,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2113,8 +1792,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>HD Projector line: chip 'Partial'. 3 total − 0 in maintenance − 2 reserved elsewhere = 1 available for these dates. 2 requested, 1 available. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -2202,7 +1881,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2210,16 +1889,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'HD Projector': 3 total, 0 in maintenance.
-Event 'Board Meeting' (2026-10-26) holds 2x HD Projector.
-Event 'Year-End Gala' (2027-01-15) requests 3x HD Projector with no other holds near that date.
+          <t>Rule source: customer Q&amp;A #82 (no maximum reservation period).
+'Lighting Rig': 1 total, 0 in maintenance.
+Event 'Three-Day Expo' (2026-11-16 to 2026-11-18, 09:00 on the first day to 17:00 on the last) holds one reservation for 1x Lighting Rig for the whole period: blocked from 2026-11-15 through its Return Day (2026-11-18), available again from 2026-11-19.
+Event 'Post-Expo Mixer' (2026-11-19) and event 'Later Concert' (2026-11-20) each request 1x Lighting Rig.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2228,8 +1908,11 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Year-End Gala event
-3. Read the HD Projector line under Requested items</t>
+2. Open the equipment request for the Post-Expo Mixer event
+3. Read the Lighting Rig line under Requested items
+4. Click Equipment Requests in the side menu
+5. Open the equipment request for the Later Concert event
+6. Read the Lighting Rig line under Requested items</t>
         </is>
       </c>
     </row>
@@ -2241,11 +1924,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: HD Projector, Requested: 3, Event date: 2027-01-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Equipment: Lighting Rig, Requested: 1, Expo: 2026-11-16 to 2026-11-18, Checked dates: 2026-11-19 and 2026-11-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2253,8 +1936,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The HD Projector line shows the chip 'Available' and '3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates'; the October hold has no effect.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>Post-Expo Mixer: the Lighting Rig line shows the chip 'Unavailable', '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates' and 'Held by Three-Day Expo (1 unit) until 19 Nov.'
+Later Concert: the Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
         </is>
       </c>
     </row>
@@ -2280,7 +1963,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2298,7 +1980,9 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>HD Projector line: chip 'Available'. 3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>[Post-Expo Mixer] Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Three-Day Expo (1 unit) until 19 Nov. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.
+[Later Concert] Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -2387,7 +2071,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="179.5" customHeight="1">
+    <row r="3" ht="220" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2395,10 +2079,10 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: SCHEMA_REFERENCE.md - only 'reserved' and 'partially_fulfilled' count against availability.
-'HD Projector': 3 total, 0 in maintenance.
-Event 'Staff Retreat' (2026-12-14) has a request for 2x HD Projector with status 'Under review' (not reserved).
-Event 'Board Meeting 2' (2026-12-14) requests 3x HD Projector.
+          <t>Rule source: customer Q&amp;A #2 (transfer time affects pre-event availability; Return Day+1 governs post-event availability). Return Day is the event's own end date; no extra time is added after the event.
+'Lighting Rig': 1 total, 0 in maintenance.
+Event 'Late Gala' (Monday 2026-11-23, 19:00-23:30) holds 1x Lighting Rig; Return Day is 2026-11-23, available again from 2026-11-24.
+Event 'Wednesday Fair' (2026-11-25) requests 1x Lighting Rig; its own D-1 is 2026-11-24.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -2414,8 +2098,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Board Meeting 2 event
-3. Read the HD Projector line under Requested items</t>
+2. Open the equipment request for the Wednesday Fair event
+3. Read the Lighting Rig line under Requested items</t>
         </is>
       </c>
     </row>
@@ -2427,11 +2111,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: HD Projector, Requested: 3, Total: 3, Other request: 2 (Under review)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Equipment: Lighting Rig, Requested: 1, Late Gala ends: 23:30 Monday, Checked date: 2026-11-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2439,7 +2123,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The HD Projector line shows the chip 'Available' and '3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates'.
+          <t>The Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates' - finishing at 23:30 does not move the Return Day to Tuesday.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -2466,7 +2150,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2484,7 +2167,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>HD Projector line: chip 'Available'. 3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -2509,7 +2192,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. Rule from SCHEMA_REFERENCE.md.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
         </is>
       </c>
     </row>
@@ -2581,10 +2264,10 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: SCHEMA_REFERENCE.md - 'partially_fulfilled' counts against availability.
-'Conference Phone': 5 total, 0 in maintenance.
-Event 'Open Day' (2026-11-06) requested 4x Conference Phone but only 2 were reserved (status 'Partially fulfilled').
-Event 'Alumni Mixer' (2026-11-06) requests 3x Conference Phone.
+          <t>Rule source: customer Q&amp;A #5 (equipment cannot be shared between events on the same day).
+'Lighting Rig': 1 total, 0 in maintenance.
+Event 'Morning Workshop' (2026-12-01, 09:00-12:00) holds 1x Lighting Rig.
+Event 'Evening Recital' (2026-12-01, 18:00-21:00, does not overlap Morning Workshop) requests 1x Lighting Rig.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -2600,8 +2283,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Alumni Mixer event
-3. Read the Conference Phone line under Requested items</t>
+2. Open the equipment request for the Evening Recital event
+3. Read the Lighting Rig line under Requested items</t>
         </is>
       </c>
     </row>
@@ -2613,11 +2296,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Conference Phone, Requested: 3, Total: 5, Open Day requested 4 / reserved 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: Lighting Rig, Requested: 1, Morning Workshop 09:00-12:00, Evening Recital 18:00-21:00, same day</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2625,8 +2308,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Conference Phone line shows the chip 'Available' and '5 total − 0 in maintenance − 2 reserved elsewhere = 3 available for these dates' - 2 (the quantity reserved), not 4 (the quantity requested).
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The Lighting Rig line shows the chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
+The line notes 'Held by Morning Workshop (1 unit) until 2 Dec.'
+The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2336,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2670,8 +2353,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Conference Phone line: chip 'Available'. 5 total − 0 in maintenance − 2 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Morning Workshop (1 unit) until 2 Dec. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
     </row>
@@ -2695,7 +2378,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. Rule from SCHEMA_REFERENCE.md.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2442,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="206.5" customHeight="1">
+    <row r="3" ht="152.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2767,10 +2450,9 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: briefing and SPM-37 (cancelling an event releases its equipment reservations). Until SPM-37 ships, the check ignores requests of cancelled events (temporary filter).
-'Presenter Tablet': 2 total, 0 in maintenance.
-Event 'Cancelled Summit' (2026-11-12) has status 'Cancelled' and its request for 2x Presenter Tablet is still marked 'Reserved'.
-Event 'Product Demo' (2026-11-12) requests 2x Presenter Tablet.
+          <t>'Stage Wash Light': 2 total, 0 in maintenance.
+Event 'Morning Workshop' (2026-12-01, 09:00-12:00) holds 1x Stage Wash Light.
+Event 'Evening Recital' (2026-12-01, 18:00-21:00) requests 1x Stage Wash Light.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -2786,8 +2468,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Product Demo event
-3. Read the Presenter Tablet line under Requested items</t>
+2. Open the equipment request for the Evening Recital event
+3. Read the Stage Wash Light line under Requested items</t>
         </is>
       </c>
     </row>
@@ -2799,11 +2481,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Presenter Tablet, Requested: 2, Total: 2, Cancelled Summit reserved: 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: Stage Wash Light, Requested: 1, Total: 2, Held by Morning Workshop: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2811,8 +2493,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Presenter Tablet line shows the chip 'Available' and '2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates' - the cancelled event's units are not counted.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The Stage Wash Light line shows the chip 'Available' and '2 total − 0 in maintenance − 1 reserved elsewhere = 1 available for these dates'.</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2519,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2856,8 +2536,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Presenter Tablet line: chip 'Available'. 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>Stage Wash Light line: chip 'Available'. 2 total − 0 in maintenance − 1 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
     </row>
@@ -2881,7 +2561,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. The cancelled-event filter is temporary until SPM-37 (Cancel Event) releases the reservation itself.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2625,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="220" customHeight="1">
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2953,17 +2633,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #5 (collected one day before the event, available again from Return Day+1). Return Day is the day the event ends.
-'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Gala Dinner' (Monday 2026-11-02, 10:00-16:00) holds 1x Lighting Rig: blocked from its D-1 (2026-11-01) through its Return Day (2026-11-02).
-Event 'Charity Concert' (Tuesday 2026-11-03) requests 1x Lighting Rig. It would need collecting on 2026-11-02 (its own D-1), while the rig is still being returned and checked.
+          <t>Rule source: customer Q&amp;A #74 (different sessions can have different equipment) and SPM-47.
+'PA Speaker': 2 total, 0 in maintenance.
+Event 'Open House' (2026-10-05) holds 2x PA Speaker.
+Event 'Two-Day Summit' has session 'Day 1' (2026-10-05) and session 'Day 2' (2026-10-20). Each session requests 2x PA Speaker.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2972,8 +2652,9 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Charity Concert event
-3. Read the Lighting Rig line under Requested items</t>
+2. Open the equipment request for the Two-Day Summit event
+3. Read the PA Speaker line under Day 1
+4. Read the PA Speaker line under Day 2</t>
         </is>
       </c>
     </row>
@@ -2985,11 +2666,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Checked date: 2026-11-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Equipment: PA Speaker, Requested: 2 per session, Day 1: 2026-10-05, Day 2: 2026-10-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2997,8 +2678,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Lighting Rig line shows the chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
-The line notes 'Held by Gala Dinner (1 unit) until 3 Nov.' (the day it is available again, Return Day+1).
+          <t>Day 1: the PA Speaker line shows the chip 'Unavailable' and '2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates'.
+Day 2: the PA Speaker line shows the chip 'Available' and '2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates'.
 The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
@@ -3025,7 +2706,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3043,7 +2723,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Gala Dinner (1 unit) until 3 Nov. Venue not yet chosen — transfer time not included.
+          <t>PA Speaker · Day 1 line: chip 'Unavailable'. 2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates. Held by Open House (2 units) until 6 Oct. Venue not yet chosen — transfer time not included.
+PA Speaker · Day 2 line: chip 'Available'. 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates. Venue not yet chosen — transfer time not included.
 Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
@@ -3132,7 +2813,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="152.5" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3140,12 +2821,10 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Gala Dinner' (Monday 2026-11-02) holds 1x Lighting Rig; it is available again from Return Day+1 (2026-11-03).
-Event 'School Concert' (Wednesday 2026-11-04) requests 1x Lighting Rig; its own D-1 is 2026-11-03.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
+          <t>Rule source: customer Q&amp;A #2 - transfer and preparation time is considered when equipment must move to the event venue. Fixed at 2 hours (team proposal).
+'Follow Spot': 1 total, 0 in maintenance, kept in ConnectSphere storage (no venue set).
+Event 'Product Showcase' (2026-10-21, 11:00-15:00) is booked at Marina Auditorium and requests 1x Follow Spot.
+This event has a venue, so it does not show 'Venue not yet chosen'.</t>
         </is>
       </c>
     </row>
@@ -3158,12 +2837,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the School Concert event
-3. Read the Lighting Rig line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Open the equipment request for the Product Showcase event
+3. Read the Follow Spot line under Requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3171,11 +2850,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Checked date: 2026-11-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Event start: 2026-10-21 11:00, Equipment location: ConnectSphere storage, Event venue: Marina Auditorium, Transfer/prep time: 2 hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3183,8 +2862,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The line shows 'Leaves 21 Oct 2026, 09:00 — 2 hours before the event for transfer and preparation.'
+The Follow Spot line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
         </is>
       </c>
     </row>
@@ -3210,7 +2889,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3228,7 +2906,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Follow Spot line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Leaves 21 Oct 2026, 09:00 — 2 hours before the event for transfer and preparation.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -3317,7 +2995,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="166" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3325,16 +3003,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Workshop Wrap-up' (Wednesday 2026-11-11) holds 1x Lighting Rig; it is collected on 2026-11-10 (D-1).
-Event 'Setup Day Talk' (Tuesday 2026-11-10) requests 1x Lighting Rig; its own Return Day (2026-11-10) runs into Workshop Wrap-up's collection day.
+          <t>'Marina Hall Sound System': 1 total, 0 in maintenance, kept at Marina Grand Hall.
+Event 'Welcome Assembly' (2026-10-21, 11:00-15:00) is booked at Marina Grand Hall and requests 1x Marina Hall Sound System.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3343,8 +3019,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Setup Day Talk event
-3. Read the Lighting Rig line under Requested items</t>
+2. Open the equipment request for the Welcome Assembly event
+3. Read the Marina Hall Sound System line under Requested items</t>
         </is>
       </c>
     </row>
@@ -3356,11 +3032,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Checked date: 2026-11-10</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Event start: 2026-10-21 11:00, Equipment location: Marina Grand Hall, Event venue: Marina Grand Hall</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3368,9 +3044,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Lighting Rig line shows the chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
-The line notes 'Held by Workshop Wrap-up (1 unit) until 12 Nov.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The line shows 'Already at the venue: needed from 21 Oct 2026, 11:00.' - no transfer or preparation time is added.
+The line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3071,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3414,8 +3088,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Workshop Wrap-up (1 unit) until 12 Nov. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>Marina Hall Sound System line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Already at the venue: needed from 21 Oct 2026, 11:00.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3177,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="220" customHeight="1">
+    <row r="3" ht="152.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3511,17 +3185,15 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #82 (no maximum reservation period).
-'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Three-Day Expo' (2026-11-16 to 2026-11-18, 09:00 on the first day to 17:00 on the last) holds one reservation for 1x Lighting Rig for the whole period: blocked from 2026-11-15 through its Return Day (2026-11-18), available again from 2026-11-19.
-Event 'Post-Expo Mixer' (2026-11-19) and event 'Later Concert' (2026-11-20) each request 1x Lighting Rig.
+          <t>'Podium Mic': 1 total, 0 in maintenance, kept in ConnectSphere storage; held on 2026-10-20 by 'Keynote Rehearsal', far from this event.
+Event 'Planning Workshop' (2026-11-03, 11:00-15:00) has no venue booked yet and requests 1x Podium Mic.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3530,15 +3202,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Post-Expo Mixer event
-3. Read the Lighting Rig line under Requested items
-4. Click Equipment Requests in the side menu
-5. Open the equipment request for the Later Concert event
-6. Read the Lighting Rig line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Open the equipment request for the Planning Workshop event
+3. Read the Podium Mic line under Requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -3546,11 +3215,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Expo: 2026-11-16 to 2026-11-18, Checked dates: 2026-11-19 and 2026-11-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Equipment: Podium Mic, Requested: 1, Event venue: none yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3558,8 +3227,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Post-Expo Mixer: the Lighting Rig line shows the chip 'Unavailable', '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates' and 'Held by Three-Day Expo (1 unit) until 19 Nov.'
-Later Concert: the Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
+          <t>The Podium Mic line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.
+The line notes 'Venue not yet chosen — transfer time not included.' No transfer time is applied.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -3585,7 +3255,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3603,9 +3272,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>[Post-Expo Mixer] Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Three-Day Expo (1 unit) until 19 Nov. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.
-[Later Concert] Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Podium Mic line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -3694,7 +3361,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="166" customHeight="1">
+    <row r="3" ht="125.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3702,9 +3369,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Cordless Mic Set': 5 total, 0 in maintenance, none reserved elsewhere.
-'Podium Mic': 1 total, held in full by 'Keynote Rehearsal' on the same day (2026-10-20).
-Event 'Town Hall Q4' (2026-10-20) requests 2x Cordless Mic Set only.
+          <t>'Smoke Machine': 0 total, 0 in maintenance.
+Event 'Halloween Party' (2026-10-30) requests 1x Smoke Machine.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -3720,8 +3386,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Town Hall Q4 event
-3. Read the Cordless Mic Set line under Requested items</t>
+2. Open the equipment request for the Halloween Party event
+3. Read the Smoke Machine line under Requested items</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3399,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Cordless Mic Set, Requested: 2</t>
+          <t>Equipment: Smoke Machine, Total: 0, Requested: 1</t>
         </is>
       </c>
     </row>
@@ -3745,9 +3411,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Cordless Mic Set line shows the chip 'Available' and '5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates'.
-Podium Mic being fully held has no effect on this line.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The Smoke Machine line shows the chip 'Unavailable' and '0 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates'.
+The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
     </row>
@@ -3773,7 +3438,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3791,8 +3455,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Cordless Mic Set line: chip 'Available'. 5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>Smoke Machine line: chip 'Unavailable'. 0 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3544,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="220" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3888,10 +3552,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #2 (transfer time affects pre-event availability; Return Day+1 governs post-event availability). Return Day is the event's own end date; no extra time is added after the event.
-'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Late Gala' (Monday 2026-11-23, 19:00-23:30) holds 1x Lighting Rig; Return Day is 2026-11-23, available again from 2026-11-24.
-Event 'Wednesday Fair' (2026-11-25) requests 1x Lighting Rig; its own D-1 is 2026-11-24.
+          <t>'Document Camera': 5 total with 2 recorded as in maintenance, none reserved elsewhere.
+Event 'Alumni Talk' (2026-10-28) requests 3x Document Camera.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -3907,8 +3569,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Wednesday Fair event
-3. Read the Lighting Rig line under Requested items</t>
+2. Open the equipment request for the Alumni Talk event
+3. Read the Document Camera line under Requested items</t>
         </is>
       </c>
     </row>
@@ -3920,11 +3582,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Late Gala ends: 23:30 Monday, Checked date: 2026-11-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: Document Camera, Total: 5, In maintenance: 2, Requested: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3932,7 +3594,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Lighting Rig line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates' - finishing at 23:30 does not move the Return Day to Tuesday.
+          <t>The Document Camera line shows the chip 'Available' and '5 total − 2 in maintenance − 0 reserved elsewhere = 3 available for these dates'.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -3959,7 +3621,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -3977,7 +3638,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Lighting Rig line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Document Camera line: chip 'Available'. 5 total − 2 in maintenance − 0 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -4066,7 +3727,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="179.5" customHeight="1">
+    <row r="3" ht="152.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4074,17 +3735,16 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #5 (equipment cannot be shared between events on the same day).
-'Lighting Rig': 1 total, 0 in maintenance.
-Event 'Morning Workshop' (2026-12-01, 09:00-12:00) holds 1x Lighting Rig.
-Event 'Evening Recital' (2026-12-01, 18:00-21:00, does not overlap Morning Workshop) requests 1x Lighting Rig.
+          <t>'Laser Pointer': 10 total but retired (inactive).
+Event 'Debate Finals' (2026-11-05) already has a request for 1x Laser Pointer.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'
+For the last two steps, log in as the assigned Coordinator, daniel.tan@connectsphere.com (password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4093,8 +3753,10 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Evening Recital event
-3. Read the Lighting Rig line under Requested items</t>
+2. Open the equipment request for the Debate Finals event
+3. Read the Laser Pointer line under Requested items
+4. Log out and log in as daniel.tan@connectsphere.com
+5. Open the Debate Finals event's Equipment page and open the Add equipment list</t>
         </is>
       </c>
     </row>
@@ -4106,11 +3768,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Lighting Rig, Requested: 1, Morning Workshop 09:00-12:00, Evening Recital 18:00-21:00, same day</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Equipment: Laser Pointer, Total: 10, Status: inactive, Requested: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4118,9 +3780,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Lighting Rig line shows the chip 'Unavailable' and '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates'.
-The line notes 'Held by Morning Workshop (1 unit) until 2 Dec.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The Laser Pointer line shows the chip 'Unavailable' with '10 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates'.
+The banner 'Not everything requested is available.' is shown above the requested items.
+Laser Pointer is not offered in the Add equipment list.</t>
         </is>
       </c>
     </row>
@@ -4146,7 +3808,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4164,8 +3825,9 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Lighting Rig line: chip 'Unavailable'. 1 total − 0 in maintenance − 1 reserved elsewhere = 0 available for these dates. Held by Morning Workshop (1 unit) until 2 Dec. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>Laser Pointer line: chip 'Unavailable'. 10 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.
+Add equipment list (GET /api/equipment as the Coordinator): Laser Pointer is not offered.</t>
         </is>
       </c>
     </row>
@@ -4189,7 +3851,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. The Add equipment list was checked through the API that feeds it (GET /api/equipment as the Coordinator), not on screen.</t>
         </is>
       </c>
     </row>
@@ -4253,7 +3915,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="152.5" customHeight="1">
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4261,16 +3923,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Stage Wash Light': 2 total, 0 in maintenance.
-Event 'Morning Workshop' (2026-12-01, 09:00-12:00) holds 1x Stage Wash Light.
-Event 'Evening Recital' (2026-12-01, 18:00-21:00) requests 1x Stage Wash Light.
+          <t>Event 'Vendor Networking Evening' (2026-11-15, 17:00-22:00, booked at Marina Grand Hall) requests 6x Lavalier Wireless Mic, 1x Streaming Encoder, 2x Truss Lighting Bar and 1x Marina Hall Sound System.
+Stock for those dates: Lavalier Wireless Mic 10 total, 2 in maintenance, 4 held by 'Regional Tech Expo' (2026-11-14). Streaming Encoder 3 total, 2 held by 'Regional Tech Expo' and 1 by 'Annual Partner Awards Night' (2026-11-16). Truss Lighting Bar 6 total, 1 in maintenance. Marina Hall Sound System 1 total, kept at Marina Grand Hall.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4279,12 +3939,13 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Evening Recital event
-3. Read the Stage Wash Light line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
+2. Open the equipment request for the Vendor Networking Evening event
+3. Read all four lines under Requested items
+4. Read the area above the requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -4292,11 +3953,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Stage Wash Light, Requested: 1, Total: 2, Held by Morning Workshop: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Lavalier Wireless Mic: requested 6, available 4. Streaming Encoder: requested 1, available 0. Truss Lighting Bar: requested 2, available 5. Marina Hall Sound System: requested 1, available 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="233.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4304,7 +3965,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Stage Wash Light line shows the chip 'Available' and '2 total − 0 in maintenance − 1 reserved elsewhere = 1 available for these dates'.</t>
+          <t>Lavalier Wireless Mic shows the chip 'Partial', '10 total − 2 in maintenance − 4 reserved elsewhere = 4 available for these dates' and '6 requested, 4 available.'
+Streaming Encoder shows the chip 'Unavailable', '3 total − 0 in maintenance − 3 reserved elsewhere = 0 available for these dates', 'Held by Regional Tech Expo (2 units) until 15 Nov.' and 'Held by Annual Partner Awards Night (1 unit) until 17 Nov.'
+Truss Lighting Bar shows the chip 'Available' and '6 total − 1 in maintenance − 0 reserved elsewhere = 5 available for these dates'.
+Marina Hall Sound System shows the chip 'Available', '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates' and 'Already at the venue: needed from 15 Nov 2026, 17:00.'
+The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
     </row>
@@ -4330,7 +3995,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -4348,1305 +4012,11 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Stage Wash Light line: chip 'Available'. 2 total − 0 in maintenance − 1 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Lavalier Wireless Mic line: chip 'Partial'. 10 total − 2 in maintenance − 4 reserved elsewhere = 4 available for these dates. 6 requested, 4 available. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
+Streaming Encoder line: chip 'Unavailable'. 3 total − 0 in maintenance − 3 reserved elsewhere = 0 available for these dates. Held by Regional Tech Expo (2 units) until 15 Nov. Held by Annual Partner Awards Night (1 unit) until 17 Nov. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
+Truss Lighting Bar line: chip 'Available'. 6 total − 1 in maintenance − 0 reserved elsewhere = 5 available for these dates. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
+Marina Hall Sound System line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Already at the venue: needed from 15 Nov 2026, 17:00.
 Banner 'Not everything requested is available.' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC22</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="179.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Rule source: customer Q&amp;A #74 (different sessions can have different equipment) and SPM-47.
-'PA Speaker': 2 total, 0 in maintenance.
-Event 'Open House' (2026-10-05) holds 2x PA Speaker.
-Event 'Two-Day Summit' has session 'Day 1' (2026-10-05) and session 'Day 2' (2026-10-20). Each session requests 2x PA Speaker.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Two-Day Summit event
-3. Read the PA Speaker line under Day 1
-4. Read the PA Speaker line under Day 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: PA Speaker, Requested: 2 per session, Day 1: 2026-10-05, Day 2: 2026-10-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="112" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Day 1: the PA Speaker line shows the chip 'Unavailable' and '2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates'.
-Day 2: the PA Speaker line shows the chip 'Available' and '2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates'.
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>PA Speaker · Day 1 line: chip 'Unavailable'. 2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates. Held by Open House (2 units) until 6 Oct. Venue not yet chosen — transfer time not included.
-PA Speaker · Day 2 line: chip 'Available'. 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC23</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="125.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Rule source: customer Q&amp;A #2 - transfer and preparation time is considered when equipment must move to the event venue. Fixed at 2 hours (team proposal).
-'Follow Spot': 1 total, 0 in maintenance, kept in ConnectSphere storage (no venue set).
-Event 'Product Showcase' (2026-10-21, 11:00-15:00) is booked at Marina Auditorium and requests 1x Follow Spot.
-This event has a venue, so it does not show 'Venue not yet chosen'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Product Showcase event
-3. Read the Follow Spot line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Event start: 2026-10-21 11:00, Equipment location: ConnectSphere storage, Event venue: Marina Auditorium, Transfer/prep time: 2 hours</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The line shows 'Leaves 21 Oct 2026, 09:00 — 2 hours before the event for transfer and preparation.'
-The Follow Spot line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Follow Spot line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Leaves 21 Oct 2026, 09:00 — 2 hours before the event for transfer and preparation.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC24</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="112" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Marina Hall Sound System': 1 total, 0 in maintenance, kept at Marina Grand Hall.
-Event 'Welcome Assembly' (2026-10-21, 11:00-15:00) is booked at Marina Grand Hall and requests 1x Marina Hall Sound System.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Welcome Assembly event
-3. Read the Marina Hall Sound System line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Event start: 2026-10-21 11:00, Equipment location: Marina Grand Hall, Event venue: Marina Grand Hall</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The line shows 'Already at the venue: needed from 21 Oct 2026, 11:00.' - no transfer or preparation time is added.
-The line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Marina Hall Sound System line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Already at the venue: needed from 21 Oct 2026, 11:00.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="152.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Podium Mic': 1 total, 0 in maintenance, kept in ConnectSphere storage; held on 2026-10-20 by 'Keynote Rehearsal', far from this event.
-Event 'Planning Workshop' (2026-11-03, 11:00-15:00) has no venue booked yet and requests 1x Podium Mic.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Planning Workshop event
-3. Read the Podium Mic line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: Podium Mic, Requested: 1, Event venue: none yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The Podium Mic line shows the chip 'Available' and '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates'.
-The line notes 'Venue not yet chosen — transfer time not included.' No transfer time is applied.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Podium Mic line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC26</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="139" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Document Camera': 5 total with 2 recorded as in maintenance, none reserved elsewhere.
-Event 'Alumni Talk' (2026-10-28) requests 3x Document Camera.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Alumni Talk event
-3. Read the Document Camera line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: Document Camera, Total: 5, In maintenance: 2, Requested: 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The Document Camera line shows the chip 'Available' and '5 total − 2 in maintenance − 0 reserved elsewhere = 3 available for these dates'.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Document Camera line: chip 'Available'. 5 total − 2 in maintenance − 0 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC27</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="152.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Laser Pointer': 10 total but retired (inactive).
-Event 'Debate Finals' (2026-11-05) already has a request for 1x Laser Pointer.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'
-For the last two steps, log in as the assigned Coordinator, daniel.tan@connectsphere.com (password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Debate Finals event
-3. Read the Laser Pointer line under Requested items
-4. Log out and log in as daniel.tan@connectsphere.com
-5. Open the Debate Finals event's Equipment page and open the Add equipment list</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: Laser Pointer, Total: 10, Status: inactive, Requested: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>The Laser Pointer line shows the chip 'Unavailable' with '10 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates'.
-The banner 'Not everything requested is available.' is shown above the requested items.
-Laser Pointer is not offered in the Add equipment list.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Laser Pointer line: chip 'Unavailable'. 10 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.
-Add equipment list (GET /api/equipment as the Coordinator): Laser Pointer is not offered.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. The Add equipment list was checked through the API that feeds it (GET /api/equipment as the Coordinator), not on screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="139" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Cordless Mic Set': 5 total, 0 in maintenance, none reserved elsewhere.
-Event 'Graduation Ceremony' (2026-10-29) requests 2x Cordless Mic Set (its only equipment line).
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Graduation Ceremony event
-3. Read the Cordless Mic Set line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: Cordless Mic Set, Requested: 2, Available: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>A green 'Available' chip is shown on the Cordless Mic Set line next to '5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates'.
-No 'Not everything requested is available.' banner is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Cordless Mic Set line: chip 'Available'. 5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -5734,7 +4104,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="125.5" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -5742,8 +4112,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Smoke Machine': 0 total, 0 in maintenance.
-Event 'Halloween Party' (2026-10-30) requests 1x Smoke Machine.
+          <t>'Tripod Screen': 4 total, 0 in maintenance, none reserved elsewhere.
+Event 'Product Launch' (2026-10-16) requests 4x Tripod Screen.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -5759,8 +4129,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Halloween Party event
-3. Read the Smoke Machine line under Requested items</t>
+2. Open the equipment request for the Product Launch event
+3. Read the Tripod Screen line under Requested items</t>
         </is>
       </c>
     </row>
@@ -5772,11 +4142,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Smoke Machine, Total: 0, Requested: 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: Tripod Screen, Requested: 4, Available: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -5784,8 +4154,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Smoke Machine line shows the chip 'Unavailable' and '0 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates'.
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The Tripod Screen line shows the chip 'Available' and '4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates'.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -5811,7 +4181,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -5829,382 +4198,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Smoke Machine line: chip 'Unavailable'. 0 total − 0 in maintenance − 0 reserved elsewhere = 0 available for these dates. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC29</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="139" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>'Cordless Mic Set': 5 total, 0 in maintenance, none reserved elsewhere.
-Event 'Graduation Ceremony 2' (2026-10-30) requests 6x Cordless Mic Set (its only equipment line).
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Graduation Ceremony 2 event
-3. Read the Cordless Mic Set line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Equipment: Cordless Mic Set, Requested: 6, Available: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>An amber 'Partial' chip is shown on the Cordless Mic Set line next to '5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates' and '6 requested, 5 available.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Cordless Mic Set line: chip 'Partial'. 5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates. 6 requested, 5 available. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
-  <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-48-TC30</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="179.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Event 'Vendor Networking Evening' (2026-11-15, 17:00-22:00, booked at Marina Grand Hall) requests 6x Lavalier Wireless Mic, 1x Streaming Encoder, 2x Truss Lighting Bar and 1x Marina Hall Sound System.
-Stock for those dates: Lavalier Wireless Mic 10 total, 2 in maintenance, 4 held by 'Regional Tech Expo' (2026-11-14). Streaming Encoder 3 total, 2 held by 'Regional Tech Expo' and 1 by 'Annual Partner Awards Night' (2026-11-16). Truss Lighting Bar 6 total, 1 in maintenance. Marina Hall Sound System 1 total, kept at Marina Grand Hall.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Vendor Networking Evening event
-3. Read all four lines under Requested items
-4. Read the area above the requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Lavalier Wireless Mic: requested 6, available 4. Streaming Encoder: requested 1, available 0. Truss Lighting Bar: requested 2, available 5. Marina Hall Sound System: requested 1, available 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="233.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Lavalier Wireless Mic shows the chip 'Partial', '10 total − 2 in maintenance − 4 reserved elsewhere = 4 available for these dates' and '6 requested, 4 available.'
-Streaming Encoder shows the chip 'Unavailable', '3 total − 0 in maintenance − 3 reserved elsewhere = 0 available for these dates', 'Held by Regional Tech Expo (2 units) until 15 Nov.' and 'Held by Annual Partner Awards Night (1 unit) until 17 Nov.'
-Truss Lighting Bar shows the chip 'Available' and '6 total − 1 in maintenance − 0 reserved elsewhere = 5 available for these dates'.
-Marina Hall Sound System shows the chip 'Available', '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates' and 'Already at the venue: needed from 15 Nov 2026, 17:00.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Creation Date</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="n">
-        <v>46291</v>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Lavalier Wireless Mic line: chip 'Partial'. 10 total − 2 in maintenance − 4 reserved elsewhere = 4 available for these dates. 6 requested, 4 available. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
-Streaming Encoder line: chip 'Unavailable'. 3 total − 0 in maintenance − 3 reserved elsewhere = 0 available for these dates. Held by Regional Tech Expo (2 units) until 15 Nov. Held by Annual Partner Awards Night (1 unit) until 17 Nov. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
-Truss Lighting Bar line: chip 'Available'. 6 total − 1 in maintenance − 0 reserved elsewhere = 5 available for these dates. Leaves 15 Nov 2026, 15:00 — 2 hours before the event for transfer and preparation.
-Marina Hall Sound System line: chip 'Available'. 1 total − 0 in maintenance − 0 reserved elsewhere = 1 available for these dates. Already at the venue: needed from 15 Nov 2026, 17:00.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>Tripod Screen line: chip 'Available'. 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates. Venue not yet chosen — transfer time not included.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -6300,8 +4295,8 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Cordless Mic Set': 5 total, 0 in maintenance, none reserved elsewhere.
-Event 'Career Fair' (2026-10-14) requests 3x Cordless Mic Set.
+          <t>'Tripod Screen': 4 total, 0 in maintenance, none reserved elsewhere.
+Event 'Product Launch 2' (2026-10-17) requests 5x Tripod Screen.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -6317,8 +4312,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Career Fair event
-3. Read the Cordless Mic Set line under Requested items</t>
+2. Open the equipment request for the Product Launch 2 event
+3. Read the Tripod Screen line under Requested items</t>
         </is>
       </c>
     </row>
@@ -6330,11 +4325,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Cordless Mic Set, Requested: 3, Available: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Equipment: Tripod Screen, Requested: 5, Available: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -6342,8 +4337,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Cordless Mic Set line shows the chip 'Available' and '5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates'.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The Tripod Screen line shows the chip 'Partial', '4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates' and '5 requested, 4 available.'
+The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
     </row>
@@ -6369,7 +4364,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -6387,8 +4381,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Cordless Mic Set line: chip 'Available'. 5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>Tripod Screen line: chip 'Partial'. 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates. 5 requested, 4 available. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
     </row>
@@ -6476,7 +4470,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="71.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -6484,15 +4478,13 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Cordless Mic Set': 5 total, 0 in maintenance, none reserved elsewhere.
-Event 'Career Fair 2' (2026-10-15) requests 10x Cordless Mic Set.
-Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
-Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="44.5" customHeight="1">
+          <t>Data: seeded by `npx prisma db seed`.
+Logged in as the assigned Coordinator, daniel.tan@connectsphere.com (password123).
+Event 'Career Fair' (2026-10-14) has a request for Cordless Mic Set only; 'Tripod Screen' is not yet requested for it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -6500,9 +4492,10 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Career Fair 2 event
-3. Read the Cordless Mic Set line under Requested items</t>
+          <t>1. Open the Career Fair event's Equipment page
+2. Under Add equipment, choose Tripod Screen
+3. Enter 0 in Quantity
+4. Click Add</t>
         </is>
       </c>
     </row>
@@ -6514,11 +4507,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Cordless Mic Set, Requested: 10, Available: 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: Tripod Screen, Quantity: 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -6526,8 +4519,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Cordless Mic Set line shows the chip 'Partial', '5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates' and '10 requested, 5 available.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The message 'Enter a whole number, at least 1.' is shown.
+Tripod Screen is not added and no availability result is produced for it.</t>
         </is>
       </c>
     </row>
@@ -6553,7 +4546,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -6571,8 +4563,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Cordless Mic Set line: chip 'Partial'. 5 total − 0 in maintenance − 0 reserved elsewhere = 5 available for these dates. 10 requested, 5 available. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>Not executed. The 'Enter a whole number, at least 1.' message is shown by the Add equipment form in the browser, which was not opened for this run.</t>
         </is>
       </c>
     </row>
@@ -6584,7 +4575,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Not Executed</t>
         </is>
       </c>
     </row>
@@ -6596,7 +4587,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
+          <t>Needs a manual check in the browser, logged in as the assigned Coordinator (daniel.tan@connectsphere.com).</t>
         </is>
       </c>
     </row>
@@ -6660,7 +4651,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="152.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -6668,15 +4659,16 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Tripod Screen': 4 total, 0 in maintenance, none reserved elsewhere.
-Event 'Product Launch' (2026-10-16) requests 4x Tripod Screen.
+          <t>'HD Projector': 3 total, 0 in maintenance.
+Event 'Board Meeting' (2026-10-26, 10:00-12:00) holds 2x HD Projector (reserved).
+Event 'Investor Briefing' (2026-10-26, 11:00-13:00, overlapping Board Meeting) requests 2x HD Projector.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -6685,12 +4677,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Product Launch event
-3. Read the Tripod Screen line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+2. Open the equipment request for the Investor Briefing event
+3. Read the HD Projector line under Requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -6698,11 +4690,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Tripod Screen, Requested: 4, Available: 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Equipment: HD Projector, Requested: 2, Total: 3, Reserved by overlapping event: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="98.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -6710,8 +4702,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Tripod Screen line shows the chip 'Available' and '4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates'.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>The HD Projector line shows the chip 'Partial', '3 total − 0 in maintenance − 2 reserved elsewhere = 1 available for these dates' and '2 requested, 1 available.'
+The 2 units held by Board Meeting are excluded from the available count.
+The banner 'Not everything requested is available.' is shown above the requested items.</t>
         </is>
       </c>
     </row>
@@ -6737,7 +4730,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -6755,8 +4747,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Tripod Screen line: chip 'Available'. 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates. Venue not yet chosen — transfer time not included.
-No 'Not everything requested is available.' banner is shown.</t>
+          <t>HD Projector line: chip 'Partial'. 3 total − 0 in maintenance − 2 reserved elsewhere = 1 available for these dates. 2 requested, 1 available. Venue not yet chosen — transfer time not included.
+Banner 'Not everything requested is available.' is shown.</t>
         </is>
       </c>
     </row>
@@ -6844,7 +4836,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="139" customHeight="1">
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -6852,8 +4844,10 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'Tripod Screen': 4 total, 0 in maintenance, none reserved elsewhere.
-Event 'Product Launch 2' (2026-10-17) requests 5x Tripod Screen.
+          <t>Rule source: SCHEMA_REFERENCE.md - only 'reserved' and 'partially_fulfilled' count against availability.
+'HD Projector': 3 total, 0 in maintenance.
+Event 'Staff Retreat' (2026-12-14) has a request for 2x HD Projector with status 'Under review' (not reserved).
+Event 'Board Meeting 2' (2026-12-14) requests 3x HD Projector.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
@@ -6869,12 +4863,12 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Product Launch 2 event
-3. Read the Tripod Screen line under Requested items</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+2. Open the equipment request for the Board Meeting 2 event
+3. Read the HD Projector line under Requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -6882,11 +4876,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Tripod Screen, Requested: 5, Available: 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>Equipment: HD Projector, Requested: 3, Total: 3, Other request: 2 (Under review)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -6894,8 +4888,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The Tripod Screen line shows the chip 'Partial', '4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates' and '5 requested, 4 available.'
-The banner 'Not everything requested is available.' is shown above the requested items.</t>
+          <t>The HD Projector line shows the chip 'Available' and '3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates'.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -6921,7 +4915,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -6939,8 +4932,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Tripod Screen line: chip 'Partial'. 4 total − 0 in maintenance − 0 reserved elsewhere = 4 available for these dates. 5 requested, 4 available. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.</t>
+          <t>HD Projector line: chip 'Available'. 3 total − 0 in maintenance − 0 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -6964,7 +4957,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. Rule from SCHEMA_REFERENCE.md.</t>
         </is>
       </c>
     </row>
@@ -7028,7 +5021,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -7036,13 +5029,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Data: seeded by `npx prisma db seed`.
-Logged in as the assigned Coordinator, daniel.tan@connectsphere.com (password123).
-Event 'Career Fair' (2026-10-14) has a request for Cordless Mic Set only; 'Tripod Screen' is not yet requested for it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>Rule source: SCHEMA_REFERENCE.md - 'partially_fulfilled' counts against availability.
+'Conference Phone': 5 total, 0 in maintenance.
+Event 'Open Day' (2026-11-06) requested 4x Conference Phone but only 2 were reserved (status 'Partially fulfilled').
+Event 'Alumni Mixer' (2026-11-06) requests 3x Conference Phone.
+Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
+Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
+Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -7050,14 +5047,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>1. Open the Career Fair event's Equipment page
-2. Under Add equipment, choose Tripod Screen
-3. Enter 0 in Quantity
-4. Click Add</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17.5" customHeight="1">
+          <t>1. Click Equipment Requests in the side menu
+2. Open the equipment request for the Alumni Mixer event
+3. Read the Conference Phone line under Requested items</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="31" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -7065,11 +5061,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: Tripod Screen, Quantity: 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+          <t>Equipment: Conference Phone, Requested: 3, Total: 5, Open Day requested 4 / reserved 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -7077,8 +5073,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>The message 'Enter a whole number, at least 1.' is shown.
-Tripod Screen is not added and no availability result is produced for it.</t>
+          <t>The Conference Phone line shows the chip 'Available' and '5 total − 0 in maintenance − 2 reserved elsewhere = 3 available for these dates' - 2 (the quantity reserved), not 4 (the quantity requested).
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -7104,7 +5100,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -7122,7 +5117,8 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Not executed. The 'Enter a whole number, at least 1.' message is shown by the Add equipment form in the browser, which was not opened for this run.</t>
+          <t>Conference Phone line: chip 'Available'. 5 total − 0 in maintenance − 2 reserved elsewhere = 3 available for these dates. Venue not yet chosen — transfer time not included.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -7134,7 +5130,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -7146,7 +5142,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Needs a manual check in the browser, logged in as the assigned Coordinator (daniel.tan@connectsphere.com).</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. Rule from SCHEMA_REFERENCE.md.</t>
         </is>
       </c>
     </row>
@@ -7210,7 +5206,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="152.5" customHeight="1">
+    <row r="3" ht="206.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -7218,16 +5214,17 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>'PA Speaker': 2 total, 0 in maintenance.
-Event 'Open House' (2026-10-05, 09:00-17:00) holds 2x PA Speaker (reserved).
-Event 'Orientation Day' (2026-10-05) and event 'Sports Meet' (2026-11-20) each request 2x PA Speaker.
+          <t>Rule source: briefing and SPM-37 (cancelling an event releases its equipment reservations). Until SPM-37 ships, the check ignores requests of cancelled events (temporary filter).
+'Presenter Tablet': 2 total, 0 in maintenance.
+Event 'Cancelled Summit' (2026-11-12) has status 'Cancelled' and its request for 2x Presenter Tablet is still marked 'Reserved'.
+Event 'Product Demo' (2026-11-12) requests 2x Presenter Tablet.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
 Unless a case says otherwise, the event has no venue booked yet, so each line also shows 'Venue not yet chosen — transfer time not included.'</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="85" customHeight="1">
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -7236,11 +5233,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Orientation Day event
-3. Read the PA Speaker line under Requested items
-4. Click Equipment Requests in the side menu
-5. Open the equipment request for the Sports Meet event
-6. Read the PA Speaker line under Requested items</t>
+2. Open the equipment request for the Product Demo event
+3. Read the Presenter Tablet line under Requested items</t>
         </is>
       </c>
     </row>
@@ -7252,11 +5246,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Equipment: PA Speaker, Requested: 2, Orientation Day: 2026-10-05, Sports Meet: 2026-11-20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="98.5" customHeight="1">
+          <t>Equipment: Presenter Tablet, Requested: 2, Total: 2, Cancelled Summit reserved: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -7264,8 +5258,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Orientation Day: the PA Speaker line shows the chip 'Unavailable', '2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates' and 'Held by Open House (2 units) until 6 Oct.'
-Sports Meet: the PA Speaker line shows the chip 'Available' and '2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates'.</t>
+          <t>The Presenter Tablet line shows the chip 'Available' and '2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates' - the cancelled event's units are not counted.
+No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
     </row>
@@ -7291,7 +5285,6 @@
         <v>46291</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -7309,9 +5302,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>[Orientation Day] PA Speaker line: chip 'Unavailable'. 2 total − 0 in maintenance − 2 reserved elsewhere = 0 available for these dates. Held by Open House (2 units) until 6 Oct. Venue not yet chosen — transfer time not included.
-Banner 'Not everything requested is available.' is shown.
-[Sports Meet] PA Speaker line: chip 'Available'. 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates. Venue not yet chosen — transfer time not included.
+          <t>Presenter Tablet line: chip 'Available'. 2 total − 0 in maintenance − 0 reserved elsewhere = 2 available for these dates. Venue not yet chosen — transfer time not included.
 No 'Not everything requested is available.' banner is shown.</t>
         </is>
       </c>
@@ -7336,7 +5327,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually.</t>
+          <t>The result was read from the app's API on 2026-09-26, which is the data the screen shows. How it looks on screen (colours, layout, exact wording) is to be confirmed manually. The cancelled-event filter is temporary until SPM-37 (Cancel Event) releases the reservation itself.</t>
         </is>
       </c>
     </row>

</xml_diff>